<commit_message>
Add birth-parent leave takers and births to parental_leave.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QQmMgvcnVHaPAUgzoirN18
</commit_message>
<xml_diff>
--- a/parental_leave_korea/data/parental_leave.xlsx
+++ b/parental_leave_korea/data/parental_leave.xlsx
@@ -3,40 +3,26 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="5260" yWindow="1960" windowWidth="26440" windowHeight="14480" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="14060" windowHeight="14480" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="181029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="1">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="12"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Helvetica Neue"/>
-      <family val="2"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Helvetica Neue"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -59,10 +45,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -150,19 +134,14 @@
         <t>users: 전체 육아휴직자 수(시작일 기준, 명). 출처: 국가데이터처 「육아휴직통계」 KOSIS DT_CC2024A001, 2026-09-29 다운로드. 공무원·교원 포함. 2024년은 잠정치(p). number(고용노동부 육아휴직급여 초회 수급자)와 정의가 다름.</t>
       </text>
     </comment>
-  </commentList>
-</comments>
-</file>
-
-<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>Claude</author>
-  </authors>
-  <commentList>
-    <comment ref="E1" authorId="0" shapeId="0">
+    <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>users: 전체 육아휴직자 수(시작일 기준, 명). 출처: 국가데이터처 「육아휴직통계」 KOSIS DT_CC2024A001, 2026-09-29 다운로드. 공무원·교원 포함. 2024년은 잠정치(p). number(고용노동부 육아휴직급여 초회 수급자)와 정의가 다름.</t>
+        <t>number3: 출생아 부모 중 육아휴직자 수(명). 그해 태어난 아이의 부모 중 같은 해 육아휴직을 시작한 사람. 출처: 국가데이터처 「육아휴직통계」 KOSIS DT_CC2024B002, 2026-09-29 다운로드. 2024년 잠정치(p). pct의 분자에 해당.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>births: 출생아 수(명). female==2(전체) 행에만 입력. 출처: KOSIS DT_CC2024B002(육아휴직통계 표에 함께 수록), 2026-09-29 다운로드.</t>
       </text>
     </comment>
   </commentList>
@@ -490,1150 +469,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>year</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>number</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>female</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>pct</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>users</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>2001</v>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>2002</v>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>3685</v>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>2003</v>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>6712</v>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>2004</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>9123</v>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>2005</v>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>10492</v>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>2006</v>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>13440</v>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>2007</v>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>20875</v>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>2008</v>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>28790</v>
-      </c>
-      <c r="C9" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>2009</v>
-      </c>
-      <c r="B10" s="2" t="n">
-        <v>34898</v>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>2010</v>
-      </c>
-      <c r="B11" s="2" t="n">
-        <v>40914</v>
-      </c>
-      <c r="C11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D11" s="2" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="E11" s="2" t="n">
-        <v>71000</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="n">
-        <v>2011</v>
-      </c>
-      <c r="B12" s="2" t="n">
-        <v>56735</v>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D12" s="2" t="n">
-        <v>46.7</v>
-      </c>
-      <c r="E12" s="2" t="n">
-        <v>90842</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>2012</v>
-      </c>
-      <c r="B13" s="2" t="n">
-        <v>62281</v>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" s="2" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="E13" s="2" t="n">
-        <v>101305</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="n">
-        <v>2013</v>
-      </c>
-      <c r="B14" s="2" t="n">
-        <v>67325</v>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="E14" s="2" t="n">
-        <v>106585</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="n">
-        <v>2014</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>73410</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="2" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="E15" s="2" t="n">
-        <v>118098</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B16" s="2" t="n">
-        <v>82467</v>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="2" t="n">
-        <v>59.1</v>
-      </c>
-      <c r="E16" s="2" t="n">
-        <v>128340</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>82179</v>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="2" t="n">
-        <v>60.4</v>
-      </c>
-      <c r="E17" s="2" t="n">
-        <v>128438</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>78080</v>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>62.2</v>
-      </c>
-      <c r="E18" s="2" t="n">
-        <v>123878</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>81537</v>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="2" t="n">
-        <v>62.9</v>
-      </c>
-      <c r="E19" s="2" t="n">
-        <v>128679</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B20" s="2" t="n">
-        <v>82868</v>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="2" t="n">
-        <v>64.59999999999999</v>
-      </c>
-      <c r="E20" s="2" t="n">
-        <v>131205</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="1" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B21" s="2" t="n">
-        <v>84617</v>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="2" t="n">
-        <v>65.7</v>
-      </c>
-      <c r="E21" s="2" t="n">
-        <v>133146</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B22" s="2" t="n">
-        <v>81514</v>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="2" t="n">
-        <v>66.90000000000001</v>
-      </c>
-      <c r="E22" s="2" t="n">
-        <v>132913</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B23" s="2" t="n">
-        <v>93200</v>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="2" t="n">
-        <v>71.09999999999999</v>
-      </c>
-      <c r="E23" s="2" t="n">
-        <v>147528</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B24" s="2" t="n">
-        <v>90672</v>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="2" t="n">
-        <v>73.2</v>
-      </c>
-      <c r="E24" s="2" t="n">
-        <v>147403</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B25" s="2" t="n">
-        <v>90706</v>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="2" t="n">
-        <v>72.2</v>
-      </c>
-      <c r="E25" s="2" t="n">
-        <v>146109</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B26" s="2" t="n">
-        <v>117129</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>2001</v>
-      </c>
-      <c r="B27" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="n">
-        <v>2002</v>
-      </c>
-      <c r="B28" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="n">
-        <v>2003</v>
-      </c>
-      <c r="B29" s="2" t="n">
-        <v>104</v>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="n">
-        <v>2004</v>
-      </c>
-      <c r="B30" s="2" t="n">
-        <v>181</v>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="n">
-        <v>2005</v>
-      </c>
-      <c r="B31" s="2" t="n">
-        <v>208</v>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="1" t="n">
-        <v>2006</v>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>230</v>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="1" t="n">
-        <v>2007</v>
-      </c>
-      <c r="B33" s="2" t="n">
-        <v>310</v>
-      </c>
-      <c r="C33" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="n">
-        <v>2008</v>
-      </c>
-      <c r="B34" s="2" t="n">
-        <v>355</v>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="1" t="n">
-        <v>2009</v>
-      </c>
-      <c r="B35" s="2" t="n">
-        <v>502</v>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="n">
-        <v>2010</v>
-      </c>
-      <c r="B36" s="2" t="n">
-        <v>819</v>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="2" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E36" s="2" t="n">
-        <v>1967</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>2011</v>
-      </c>
-      <c r="B37" s="2" t="n">
-        <v>1402</v>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D37" s="2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E37" s="2" t="n">
-        <v>3053</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>2012</v>
-      </c>
-      <c r="B38" s="2" t="n">
-        <v>1790</v>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="2" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E38" s="2" t="n">
-        <v>3691</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>2013</v>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>2293</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="2" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="E39" s="2" t="n">
-        <v>4498</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="n">
-        <v>2014</v>
-      </c>
-      <c r="B40" s="2" t="n">
-        <v>3421</v>
-      </c>
-      <c r="C40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D40" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="E40" s="2" t="n">
-        <v>6219</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B41" s="2" t="n">
-        <v>4872</v>
-      </c>
-      <c r="C41" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" s="2" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="E41" s="2" t="n">
-        <v>8220</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B42" s="2" t="n">
-        <v>7616</v>
-      </c>
-      <c r="C42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="2" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E42" s="2" t="n">
-        <v>11965</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B43" s="2" t="n">
-        <v>12042</v>
-      </c>
-      <c r="C43" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D43" s="2" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="E43" s="2" t="n">
-        <v>18160</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B44" s="2" t="n">
-        <v>17662</v>
-      </c>
-      <c r="C44" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D44" s="2" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="E44" s="2" t="n">
-        <v>25062</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B45" s="2" t="n">
-        <v>22297</v>
-      </c>
-      <c r="C45" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D45" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="E45" s="2" t="n">
-        <v>32051</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B46" s="2" t="n">
-        <v>27421</v>
-      </c>
-      <c r="C46" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="2" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="E46" s="2" t="n">
-        <v>38813</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B47" s="2" t="n">
-        <v>29041</v>
-      </c>
-      <c r="C47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D47" s="2" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>42197</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B48" s="2" t="n">
-        <v>37884</v>
-      </c>
-      <c r="C48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D48" s="2" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="E48" s="2" t="n">
-        <v>54565</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B49" s="2" t="n">
-        <v>35336</v>
-      </c>
-      <c r="C49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D49" s="2" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="E49" s="2" t="n">
-        <v>50815</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B50" s="2" t="n">
-        <v>41829</v>
-      </c>
-      <c r="C50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D50" s="2" t="n">
-        <v>10.2</v>
-      </c>
-      <c r="E50" s="2" t="n">
-        <v>60117</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
-        <v>2025</v>
-      </c>
-      <c r="B51" s="2" t="n">
-        <v>67200</v>
-      </c>
-      <c r="C51" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="n">
-        <v>2001</v>
-      </c>
-      <c r="B52" s="2">
-        <f>SUM(B2,B27)</f>
-        <v>25</v>
-      </c>
-      <c r="C52" s="2" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>2002</v>
-      </c>
-      <c r="B53" s="2">
-        <f>SUM(B3,B28)</f>
-        <v>3763</v>
-      </c>
-      <c r="C53" s="2" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="n">
-        <v>2003</v>
-      </c>
-      <c r="B54" s="2">
-        <f>SUM(B4,B29)</f>
-        <v>6816</v>
-      </c>
-      <c r="C54" s="2" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="n">
-        <v>2004</v>
-      </c>
-      <c r="B55" s="2">
-        <f>SUM(B5,B30)</f>
-        <v>9304</v>
-      </c>
-      <c r="C55" s="2" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="n">
-        <v>2005</v>
-      </c>
-      <c r="B56" s="2">
-        <f>SUM(B6,B31)</f>
-        <v>10700</v>
-      </c>
-      <c r="C56" s="2" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="n">
-        <v>2006</v>
-      </c>
-      <c r="B57" s="2">
-        <f>SUM(B7,B32)</f>
-        <v>13670</v>
-      </c>
-      <c r="C57" s="2" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="n">
-        <v>2007</v>
-      </c>
-      <c r="B58" s="2">
-        <f>SUM(B8,B33)</f>
-        <v>21185</v>
-      </c>
-      <c r="C58" s="2" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="n">
-        <v>2008</v>
-      </c>
-      <c r="B59" s="2">
-        <f>SUM(B9,B34)</f>
-        <v>29145</v>
-      </c>
-      <c r="C59" s="2" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="n">
-        <v>2009</v>
-      </c>
-      <c r="B60" s="2">
-        <f>SUM(B10,B35)</f>
-        <v>35400</v>
-      </c>
-      <c r="C60" s="2" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="n">
-        <v>2010</v>
-      </c>
-      <c r="B61" s="2">
-        <f>SUM(B11,B36)</f>
-        <v>41733</v>
-      </c>
-      <c r="C61" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D61" s="2" t="n">
-        <v>11.9</v>
-      </c>
-      <c r="E61" s="2" t="n">
-        <v>72967</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>2011</v>
-      </c>
-      <c r="B62" s="2">
-        <f>SUM(B12,B37)</f>
-        <v>58137</v>
-      </c>
-      <c r="C62" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D62" s="2" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="E62" s="2" t="n">
-        <v>93895</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="n">
-        <v>2012</v>
-      </c>
-      <c r="B63" s="2">
-        <f>SUM(B13,B38)</f>
-        <v>64071</v>
-      </c>
-      <c r="C63" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D63" s="2" t="n">
-        <v>15.2</v>
-      </c>
-      <c r="E63" s="2" t="n">
-        <v>104996</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="1" t="n">
-        <v>2013</v>
-      </c>
-      <c r="B64" s="2">
-        <f>SUM(B14,B39)</f>
-        <v>69618</v>
-      </c>
-      <c r="C64" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D64" s="2" t="n">
-        <v>16.4</v>
-      </c>
-      <c r="E64" s="2" t="n">
-        <v>111083</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="n">
-        <v>2014</v>
-      </c>
-      <c r="B65" s="2">
-        <f>SUM(B15,B40)</f>
-        <v>76831</v>
-      </c>
-      <c r="C65" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D65" s="2" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="E65" s="2" t="n">
-        <v>124317</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="1" t="n">
-        <v>2015</v>
-      </c>
-      <c r="B66" s="2">
-        <f>SUM(B16,B41)</f>
-        <v>87339</v>
-      </c>
-      <c r="C66" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D66" s="2" t="n">
-        <v>19.1</v>
-      </c>
-      <c r="E66" s="2" t="n">
-        <v>136560</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="n">
-        <v>2016</v>
-      </c>
-      <c r="B67" s="2">
-        <f>SUM(B17,B42)</f>
-        <v>89795</v>
-      </c>
-      <c r="C67" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D67" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="E67" s="2" t="n">
-        <v>140403</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="n">
-        <v>2017</v>
-      </c>
-      <c r="B68" s="2">
-        <f>SUM(B18,B43)</f>
-        <v>90122</v>
-      </c>
-      <c r="C68" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D68" s="2" t="n">
-        <v>21.6</v>
-      </c>
-      <c r="E68" s="2" t="n">
-        <v>142038</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="1" t="n">
-        <v>2018</v>
-      </c>
-      <c r="B69" s="2">
-        <f>SUM(B19,B44)</f>
-        <v>99199</v>
-      </c>
-      <c r="C69" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D69" s="2" t="n">
-        <v>22.5</v>
-      </c>
-      <c r="E69" s="2" t="n">
-        <v>153741</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="1" t="n">
-        <v>2019</v>
-      </c>
-      <c r="B70" s="2">
-        <f>SUM(B20,B45)</f>
-        <v>105165</v>
-      </c>
-      <c r="C70" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D70" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="E70" s="2" t="n">
-        <v>163256</v>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="1" t="n">
-        <v>2020</v>
-      </c>
-      <c r="B71" s="2">
-        <f>SUM(B21,B46)</f>
-        <v>112038</v>
-      </c>
-      <c r="C71" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D71" s="2" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="E71" s="2" t="n">
-        <v>171959</v>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="1" t="n">
-        <v>2021</v>
-      </c>
-      <c r="B72" s="2">
-        <f>SUM(B22,B47)</f>
-        <v>110555</v>
-      </c>
-      <c r="C72" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D72" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="E72" s="2" t="n">
-        <v>175110</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="1" t="n">
-        <v>2022</v>
-      </c>
-      <c r="B73" s="2">
-        <f>SUM(B23,B48)</f>
-        <v>131084</v>
-      </c>
-      <c r="C73" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D73" s="2" t="n">
-        <v>31.2</v>
-      </c>
-      <c r="E73" s="2" t="n">
-        <v>202093</v>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="1" t="n">
-        <v>2023</v>
-      </c>
-      <c r="B74" s="2">
-        <f>SUM(B24,B49)</f>
-        <v>126008</v>
-      </c>
-      <c r="C74" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D74" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="E74" s="2" t="n">
-        <v>198218</v>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="1" t="n">
-        <v>2024</v>
-      </c>
-      <c r="B75" s="2">
-        <f>SUM(B25,B50)</f>
-        <v>132535</v>
-      </c>
-      <c r="C75" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D75" s="2" t="n">
-        <v>34.7</v>
-      </c>
-      <c r="E75" s="2" t="n">
-        <v>206226</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="C76" s="2" t="n"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E75"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="4" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1644,7 +485,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>number</t>
+          <t>number1</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -1659,7 +500,17 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>users</t>
+          <t>number2</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>number3</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>births</t>
         </is>
       </c>
     </row>
@@ -1778,6 +629,9 @@
       <c r="E11" t="n">
         <v>71000</v>
       </c>
+      <c r="F11" t="n">
+        <v>47393</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1795,6 +649,9 @@
       <c r="E12" t="n">
         <v>90842</v>
       </c>
+      <c r="F12" t="n">
+        <v>57474</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1812,6 +669,9 @@
       <c r="E13" t="n">
         <v>101305</v>
       </c>
+      <c r="F13" t="n">
+        <v>65519</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1829,6 +689,9 @@
       <c r="E14" t="n">
         <v>106585</v>
       </c>
+      <c r="F14" t="n">
+        <v>65440</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1846,6 +709,9 @@
       <c r="E15" t="n">
         <v>118098</v>
       </c>
+      <c r="F15" t="n">
+        <v>70765</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1863,6 +729,9 @@
       <c r="E16" t="n">
         <v>128340</v>
       </c>
+      <c r="F16" t="n">
+        <v>76643</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1880,6 +749,9 @@
       <c r="E17" t="n">
         <v>128438</v>
       </c>
+      <c r="F17" t="n">
+        <v>74714</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1897,6 +769,9 @@
       <c r="E18" t="n">
         <v>123878</v>
       </c>
+      <c r="F18" t="n">
+        <v>69836</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1914,6 +789,9 @@
       <c r="E19" t="n">
         <v>128679</v>
       </c>
+      <c r="F19" t="n">
+        <v>69949</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1931,6 +809,9 @@
       <c r="E20" t="n">
         <v>131205</v>
       </c>
+      <c r="F20" t="n">
+        <v>69796</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1948,6 +829,9 @@
       <c r="E21" t="n">
         <v>133146</v>
       </c>
+      <c r="F21" t="n">
+        <v>67404</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1965,6 +849,9 @@
       <c r="E22" t="n">
         <v>132913</v>
       </c>
+      <c r="F22" t="n">
+        <v>69458</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1982,6 +869,9 @@
       <c r="E23" t="n">
         <v>147528</v>
       </c>
+      <c r="F23" t="n">
+        <v>75632</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1999,6 +889,9 @@
       <c r="E24" t="n">
         <v>147403</v>
       </c>
+      <c r="F24" t="n">
+        <v>76075</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2016,6 +909,9 @@
       <c r="E25" t="n">
         <v>146109</v>
       </c>
+      <c r="F25" t="n">
+        <v>79736</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2143,6 +1039,9 @@
       <c r="E36" t="n">
         <v>1967</v>
       </c>
+      <c r="F36" t="n">
+        <v>619</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2160,6 +1059,9 @@
       <c r="E37" t="n">
         <v>3053</v>
       </c>
+      <c r="F37" t="n">
+        <v>855</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -2177,6 +1079,9 @@
       <c r="E38" t="n">
         <v>3691</v>
       </c>
+      <c r="F38" t="n">
+        <v>986</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -2194,6 +1099,9 @@
       <c r="E39" t="n">
         <v>4498</v>
       </c>
+      <c r="F39" t="n">
+        <v>1089</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -2211,6 +1119,9 @@
       <c r="E40" t="n">
         <v>6219</v>
       </c>
+      <c r="F40" t="n">
+        <v>1392</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -2228,6 +1139,9 @@
       <c r="E41" t="n">
         <v>8220</v>
       </c>
+      <c r="F41" t="n">
+        <v>1752</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -2245,6 +1159,9 @@
       <c r="E42" t="n">
         <v>11965</v>
       </c>
+      <c r="F42" t="n">
+        <v>2375</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -2262,6 +1179,9 @@
       <c r="E43" t="n">
         <v>18160</v>
       </c>
+      <c r="F43" t="n">
+        <v>4126</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -2279,6 +1199,9 @@
       <c r="E44" t="n">
         <v>25062</v>
       </c>
+      <c r="F44" t="n">
+        <v>5278</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -2296,6 +1219,9 @@
       <c r="E45" t="n">
         <v>32051</v>
       </c>
+      <c r="F45" t="n">
+        <v>6340</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -2313,6 +1239,9 @@
       <c r="E46" t="n">
         <v>38813</v>
       </c>
+      <c r="F46" t="n">
+        <v>6871</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -2330,6 +1259,9 @@
       <c r="E47" t="n">
         <v>42197</v>
       </c>
+      <c r="F47" t="n">
+        <v>7933</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -2347,6 +1279,9 @@
       <c r="E48" t="n">
         <v>54565</v>
       </c>
+      <c r="F48" t="n">
+        <v>12486</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2364,6 +1299,9 @@
       <c r="E49" t="n">
         <v>50815</v>
       </c>
+      <c r="F49" t="n">
+        <v>12193</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -2381,6 +1319,9 @@
       <c r="E50" t="n">
         <v>60117</v>
       </c>
+      <c r="F50" t="n">
+        <v>17074</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -2508,6 +1449,12 @@
       <c r="E61" t="n">
         <v>72967</v>
       </c>
+      <c r="F61" t="n">
+        <v>48012</v>
+      </c>
+      <c r="G61" t="n">
+        <v>470171</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2525,6 +1472,12 @@
       <c r="E62" t="n">
         <v>93895</v>
       </c>
+      <c r="F62" t="n">
+        <v>58329</v>
+      </c>
+      <c r="G62" t="n">
+        <v>471265</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2542,6 +1495,12 @@
       <c r="E63" t="n">
         <v>104996</v>
       </c>
+      <c r="F63" t="n">
+        <v>66505</v>
+      </c>
+      <c r="G63" t="n">
+        <v>484550</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2559,6 +1518,12 @@
       <c r="E64" t="n">
         <v>111083</v>
       </c>
+      <c r="F64" t="n">
+        <v>66529</v>
+      </c>
+      <c r="G64" t="n">
+        <v>436455</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2576,6 +1541,12 @@
       <c r="E65" t="n">
         <v>124317</v>
       </c>
+      <c r="F65" t="n">
+        <v>72157</v>
+      </c>
+      <c r="G65" t="n">
+        <v>435435</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2593,6 +1564,12 @@
       <c r="E66" t="n">
         <v>136560</v>
       </c>
+      <c r="F66" t="n">
+        <v>78395</v>
+      </c>
+      <c r="G66" t="n">
+        <v>438420</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2610,6 +1587,12 @@
       <c r="E67" t="n">
         <v>140403</v>
       </c>
+      <c r="F67" t="n">
+        <v>77089</v>
+      </c>
+      <c r="G67" t="n">
+        <v>406243</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2627,6 +1610,12 @@
       <c r="E68" t="n">
         <v>142038</v>
       </c>
+      <c r="F68" t="n">
+        <v>73962</v>
+      </c>
+      <c r="G68" t="n">
+        <v>357771</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2644,6 +1633,12 @@
       <c r="E69" t="n">
         <v>153741</v>
       </c>
+      <c r="F69" t="n">
+        <v>75227</v>
+      </c>
+      <c r="G69" t="n">
+        <v>326822</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2661,6 +1656,12 @@
       <c r="E70" t="n">
         <v>163256</v>
       </c>
+      <c r="F70" t="n">
+        <v>76136</v>
+      </c>
+      <c r="G70" t="n">
+        <v>302676</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2678,6 +1679,12 @@
       <c r="E71" t="n">
         <v>171959</v>
       </c>
+      <c r="F71" t="n">
+        <v>74275</v>
+      </c>
+      <c r="G71" t="n">
+        <v>272337</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2695,6 +1702,12 @@
       <c r="E72" t="n">
         <v>175110</v>
       </c>
+      <c r="F72" t="n">
+        <v>77391</v>
+      </c>
+      <c r="G72" t="n">
+        <v>260562</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2712,6 +1725,12 @@
       <c r="E73" t="n">
         <v>202093</v>
       </c>
+      <c r="F73" t="n">
+        <v>88118</v>
+      </c>
+      <c r="G73" t="n">
+        <v>249186</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2729,6 +1748,12 @@
       <c r="E74" t="n">
         <v>198218</v>
       </c>
+      <c r="F74" t="n">
+        <v>88268</v>
+      </c>
+      <c r="G74" t="n">
+        <v>230028</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2745,6 +1770,12 @@
       </c>
       <c r="E75" t="n">
         <v>206226</v>
+      </c>
+      <c r="F75" t="n">
+        <v>96810</v>
+      </c>
+      <c r="G75" t="n">
+        <v>238317</v>
       </c>
     </row>
   </sheetData>

</xml_diff>